<commit_message>
Sidhpur Railway Station commissioned (2026)
Per the updated Completed Projects sheet: Sidhpur moves from On site to
Commissioned 2026, gets a gallery card and hero slide with its nameboard,
and its photo leaves the On site section. Totals now 14 commissioned,
8 on site; stations 10 done, 5 underway.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CqhKiE5t2z8ibPyqRLCJCS
</commit_message>
<xml_diff>
--- a/Resources/Completed projects/Completed Projects.xlsx
+++ b/Resources/Completed projects/Completed Projects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Samsung\Desktop\kivasaglobaltech.com\Resources\Completed projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEB56CD0-0D95-449A-AEA3-8801A82E6836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B870B0-BD8E-440D-98B9-8F14E73B5C8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="59">
   <si>
     <t>Project</t>
   </si>
@@ -209,6 +209,9 @@
   </si>
   <si>
     <t>Pit Lighting</t>
+  </si>
+  <si>
+    <t>Sidhpur Railway Station.jpeg</t>
   </si>
 </sst>
 </file>
@@ -1017,10 +1020,10 @@
         <v>15</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
+      </c>
+      <c r="C22" s="3">
+        <v>2026</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>51</v>
@@ -1029,7 +1032,7 @@
         <v>43</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="42.75" x14ac:dyDescent="0.45">
@@ -1069,9 +1072,10 @@
     <hyperlink ref="F9" r:id="rId13" xr:uid="{1CDD0146-38CE-4E43-9C23-3D157A0CAA89}"/>
     <hyperlink ref="F14" r:id="rId14" xr:uid="{DC0174D8-01D2-4EAF-872A-2C106AE03964}"/>
     <hyperlink ref="F15:F16" r:id="rId15" display="Under construction.png" xr:uid="{2E4802D3-EB90-4823-B4C1-1BA5C9A88029}"/>
+    <hyperlink ref="F22" r:id="rId16" xr:uid="{236E8BBA-1F66-423B-ADF5-05CB67B015E6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="63" orientation="portrait" r:id="rId16"/>
+  <pageSetup scale="63" orientation="portrait" r:id="rId17"/>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="5" min="2" max="19" man="1"/>
   </colBreaks>

</xml_diff>